<commit_message>
fix(security): scrub what review found: id-derived phones, WhatsApp ids, spreadsheets, DB password
- fixture phones built as +60 + contact id now follow the fake id (207 files)
- WhatsApp MY.<digits> per-user ids -> stable fakes (76 files)
- spreadsheet fixtures: driver and plate cells, phones and a comment scrubbed
- sorento_crm/docker-compose.yml requires POSTGRES_PASSWORD instead of a default
  (prod runs its own compose on the server)
- a doc password, a webmail address, a local DB URL and an n8n inbox id replaced
- old test fakes moved to the strict fake shape the guard now enforces
- .env.browse untracked; root *.yml snapshots ignored
- PLAN + UAC under documentation/plans/security/

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sorento_crm_frontend/e2e/fixtures/debtor-listing.xlsx
+++ b/sorento_crm_frontend/e2e/fixtures/debtor-listing.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>016-225 8620</t>
+          <t>016-000 0505</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>011-2233 4455</t>
+          <t>011-0000 0802</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>